<commit_message>
Fix: remove old dashboard.html, push_updates live stats
</commit_message>
<xml_diff>
--- a/logs/Trading_Journal.xlsx
+++ b/logs/Trading_Journal.xlsx
@@ -19,10 +19,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="₹#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="0.0&quot;%&quot;"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -62,8 +63,14 @@
       <color rgb="001E8449"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00922B21"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -115,6 +122,16 @@
         <fgColor rgb="00F2F7FC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FADBD8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F8F5"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -142,7 +159,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -190,6 +207,24 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -558,7 +593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R69"/>
+  <dimension ref="A1:R82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4829,6 +4864,828 @@
         <v>0</v>
       </c>
       <c r="R69" s="12" t="inlineStr">
+        <is>
+          <t>RSI BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="22" customHeight="1">
+      <c r="A70" s="15" t="n">
+        <v>68</v>
+      </c>
+      <c r="B70" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="C70" s="15" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="D70" s="15" t="inlineStr">
+        <is>
+          <t>AAVE-USD</t>
+        </is>
+      </c>
+      <c r="E70" s="15" t="inlineStr">
+        <is>
+          <t>CRYPTO</t>
+        </is>
+      </c>
+      <c r="F70" s="13" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G70" s="16" t="n">
+        <v>92.63</v>
+      </c>
+      <c r="H70" s="16" t="inlineStr"/>
+      <c r="I70" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="J70" s="16" t="n">
+        <v>92.63</v>
+      </c>
+      <c r="K70" s="16" t="n">
+        <v>88.9248</v>
+      </c>
+      <c r="L70" s="16" t="n">
+        <v>97.2615</v>
+      </c>
+      <c r="M70" s="16" t="inlineStr"/>
+      <c r="N70" s="15" t="inlineStr"/>
+      <c r="O70" s="15" t="n">
+        <v>29.96</v>
+      </c>
+      <c r="P70" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q70" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="R70" s="15" t="inlineStr">
+        <is>
+          <t>RSI BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="22" customHeight="1">
+      <c r="A71" s="12" t="n">
+        <v>69</v>
+      </c>
+      <c r="B71" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="C71" s="12" t="inlineStr">
+        <is>
+          <t>08:10</t>
+        </is>
+      </c>
+      <c r="D71" s="12" t="inlineStr">
+        <is>
+          <t>SOL-USD</t>
+        </is>
+      </c>
+      <c r="E71" s="12" t="inlineStr">
+        <is>
+          <t>CRYPTO</t>
+        </is>
+      </c>
+      <c r="F71" s="13" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G71" s="14" t="n">
+        <v>82.84</v>
+      </c>
+      <c r="H71" s="14" t="inlineStr"/>
+      <c r="I71" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J71" s="14" t="n">
+        <v>82.84</v>
+      </c>
+      <c r="K71" s="14" t="n">
+        <v>79.5264</v>
+      </c>
+      <c r="L71" s="14" t="n">
+        <v>86.982</v>
+      </c>
+      <c r="M71" s="14" t="inlineStr"/>
+      <c r="N71" s="12" t="inlineStr"/>
+      <c r="O71" s="12" t="n">
+        <v>29.59</v>
+      </c>
+      <c r="P71" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q71" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R71" s="12" t="inlineStr">
+        <is>
+          <t>RSI BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="22" customHeight="1">
+      <c r="A72" s="15" t="n">
+        <v>70</v>
+      </c>
+      <c r="B72" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="C72" s="15" t="inlineStr">
+        <is>
+          <t>08:10</t>
+        </is>
+      </c>
+      <c r="D72" s="15" t="inlineStr">
+        <is>
+          <t>LINK-USD</t>
+        </is>
+      </c>
+      <c r="E72" s="15" t="inlineStr">
+        <is>
+          <t>CRYPTO</t>
+        </is>
+      </c>
+      <c r="F72" s="13" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G72" s="16" t="n">
+        <v>9.074999999999999</v>
+      </c>
+      <c r="H72" s="16" t="inlineStr"/>
+      <c r="I72" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="J72" s="16" t="n">
+        <v>27.22</v>
+      </c>
+      <c r="K72" s="16" t="n">
+        <v>8.712</v>
+      </c>
+      <c r="L72" s="16" t="n">
+        <v>9.5288</v>
+      </c>
+      <c r="M72" s="16" t="inlineStr"/>
+      <c r="N72" s="15" t="inlineStr"/>
+      <c r="O72" s="15" t="n">
+        <v>28.4</v>
+      </c>
+      <c r="P72" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q72" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="R72" s="15" t="inlineStr">
+        <is>
+          <t>RSI BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="22" customHeight="1">
+      <c r="A73" s="12" t="n">
+        <v>71</v>
+      </c>
+      <c r="B73" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="C73" s="12" t="inlineStr">
+        <is>
+          <t>08:16</t>
+        </is>
+      </c>
+      <c r="D73" s="12" t="inlineStr">
+        <is>
+          <t>BNB-USD</t>
+        </is>
+      </c>
+      <c r="E73" s="12" t="inlineStr">
+        <is>
+          <t>CRYPTO</t>
+        </is>
+      </c>
+      <c r="F73" s="13" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G73" s="14" t="n">
+        <v>616.14</v>
+      </c>
+      <c r="H73" s="14" t="inlineStr"/>
+      <c r="I73" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J73" s="14" t="n">
+        <v>616.14</v>
+      </c>
+      <c r="K73" s="14" t="n">
+        <v>591.4944</v>
+      </c>
+      <c r="L73" s="14" t="n">
+        <v>646.947</v>
+      </c>
+      <c r="M73" s="14" t="inlineStr"/>
+      <c r="N73" s="12" t="inlineStr"/>
+      <c r="O73" s="12" t="n">
+        <v>29.19</v>
+      </c>
+      <c r="P73" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q73" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R73" s="12" t="inlineStr">
+        <is>
+          <t>RSI BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="22" customHeight="1">
+      <c r="A74" s="15" t="n">
+        <v>72</v>
+      </c>
+      <c r="B74" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="C74" s="15" t="inlineStr">
+        <is>
+          <t>09:19</t>
+        </is>
+      </c>
+      <c r="D74" s="15" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="E74" s="15" t="inlineStr">
+        <is>
+          <t>STOCK</t>
+        </is>
+      </c>
+      <c r="F74" s="13" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G74" s="16" t="n">
+        <v>768.4</v>
+      </c>
+      <c r="H74" s="16" t="inlineStr"/>
+      <c r="I74" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="J74" s="16" t="n">
+        <v>2305.2</v>
+      </c>
+      <c r="K74" s="16" t="n">
+        <v>753.032</v>
+      </c>
+      <c r="L74" s="16" t="n">
+        <v>791.452</v>
+      </c>
+      <c r="M74" s="16" t="inlineStr"/>
+      <c r="N74" s="15" t="inlineStr"/>
+      <c r="O74" s="15" t="n">
+        <v>14.87</v>
+      </c>
+      <c r="P74" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q74" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="R74" s="15" t="inlineStr">
+        <is>
+          <t>RSI BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="22" customHeight="1">
+      <c r="A75" s="12" t="n">
+        <v>73</v>
+      </c>
+      <c r="B75" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="C75" s="12" t="inlineStr">
+        <is>
+          <t>08:48</t>
+        </is>
+      </c>
+      <c r="D75" s="12" t="inlineStr">
+        <is>
+          <t>BNB-USD</t>
+        </is>
+      </c>
+      <c r="E75" s="12" t="inlineStr">
+        <is>
+          <t>CRYPTO</t>
+        </is>
+      </c>
+      <c r="F75" s="17" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="G75" s="14" t="n">
+        <v>52679.97</v>
+      </c>
+      <c r="H75" s="14" t="n">
+        <v>617.7</v>
+      </c>
+      <c r="I75" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J75" s="14" t="n">
+        <v>52679.97</v>
+      </c>
+      <c r="K75" s="14" t="inlineStr"/>
+      <c r="L75" s="14" t="inlineStr"/>
+      <c r="M75" s="18" t="n">
+        <v>-52062.27</v>
+      </c>
+      <c r="N75" s="17" t="inlineStr">
+        <is>
+          <t>LOSS 🔴</t>
+        </is>
+      </c>
+      <c r="O75" s="12" t="n">
+        <v>70.61</v>
+      </c>
+      <c r="P75" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q75" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R75" s="12" t="inlineStr">
+        <is>
+          <t>RSI SELL 📉</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="22" customHeight="1">
+      <c r="A76" s="15" t="n">
+        <v>74</v>
+      </c>
+      <c r="B76" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="C76" s="15" t="inlineStr">
+        <is>
+          <t>08:54</t>
+        </is>
+      </c>
+      <c r="D76" s="15" t="inlineStr">
+        <is>
+          <t>SOL-USD</t>
+        </is>
+      </c>
+      <c r="E76" s="15" t="inlineStr">
+        <is>
+          <t>CRYPTO</t>
+        </is>
+      </c>
+      <c r="F76" s="17" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="G76" s="16" t="n">
+        <v>7082.82</v>
+      </c>
+      <c r="H76" s="16" t="n">
+        <v>84.26000000000001</v>
+      </c>
+      <c r="I76" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="J76" s="16" t="n">
+        <v>7082.82</v>
+      </c>
+      <c r="K76" s="16" t="inlineStr"/>
+      <c r="L76" s="16" t="inlineStr"/>
+      <c r="M76" s="22" t="n">
+        <v>-6998.56</v>
+      </c>
+      <c r="N76" s="17" t="inlineStr">
+        <is>
+          <t>LOSS 🔴</t>
+        </is>
+      </c>
+      <c r="O76" s="15" t="n">
+        <v>76.59</v>
+      </c>
+      <c r="P76" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q76" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="R76" s="15" t="inlineStr">
+        <is>
+          <t>RSI SELL 📉</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="22" customHeight="1">
+      <c r="A77" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="B77" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="C77" s="12" t="inlineStr">
+        <is>
+          <t>08:54</t>
+        </is>
+      </c>
+      <c r="D77" s="12" t="inlineStr">
+        <is>
+          <t>LINK-USD</t>
+        </is>
+      </c>
+      <c r="E77" s="12" t="inlineStr">
+        <is>
+          <t>CRYPTO</t>
+        </is>
+      </c>
+      <c r="F77" s="17" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="G77" s="14" t="n">
+        <v>775.91</v>
+      </c>
+      <c r="H77" s="14" t="n">
+        <v>9.195</v>
+      </c>
+      <c r="I77" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="J77" s="14" t="n">
+        <v>2327.73</v>
+      </c>
+      <c r="K77" s="14" t="inlineStr"/>
+      <c r="L77" s="14" t="inlineStr"/>
+      <c r="M77" s="18" t="n">
+        <v>-2300.14</v>
+      </c>
+      <c r="N77" s="17" t="inlineStr">
+        <is>
+          <t>LOSS 🔴</t>
+        </is>
+      </c>
+      <c r="O77" s="12" t="n">
+        <v>77.76000000000001</v>
+      </c>
+      <c r="P77" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q77" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R77" s="12" t="inlineStr">
+        <is>
+          <t>RSI SELL 📉</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="22" customHeight="1">
+      <c r="A78" s="15" t="n">
+        <v>76</v>
+      </c>
+      <c r="B78" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="C78" s="15" t="inlineStr">
+        <is>
+          <t>08:54</t>
+        </is>
+      </c>
+      <c r="D78" s="15" t="inlineStr">
+        <is>
+          <t>AAVE-USD</t>
+        </is>
+      </c>
+      <c r="E78" s="15" t="inlineStr">
+        <is>
+          <t>CRYPTO</t>
+        </is>
+      </c>
+      <c r="F78" s="17" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="G78" s="16" t="n">
+        <v>7919.86</v>
+      </c>
+      <c r="H78" s="16" t="n">
+        <v>93.76000000000001</v>
+      </c>
+      <c r="I78" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="J78" s="16" t="n">
+        <v>7919.86</v>
+      </c>
+      <c r="K78" s="16" t="inlineStr"/>
+      <c r="L78" s="16" t="inlineStr"/>
+      <c r="M78" s="22" t="n">
+        <v>-7826.1</v>
+      </c>
+      <c r="N78" s="17" t="inlineStr">
+        <is>
+          <t>LOSS 🔴</t>
+        </is>
+      </c>
+      <c r="O78" s="15" t="n">
+        <v>73.53</v>
+      </c>
+      <c r="P78" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q78" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="R78" s="15" t="inlineStr">
+        <is>
+          <t>RSI SELL 📉</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="22" customHeight="1">
+      <c r="A79" s="12" t="n">
+        <v>77</v>
+      </c>
+      <c r="B79" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="C79" s="12" t="inlineStr">
+        <is>
+          <t>10:21</t>
+        </is>
+      </c>
+      <c r="D79" s="12" t="inlineStr">
+        <is>
+          <t>HG</t>
+        </is>
+      </c>
+      <c r="E79" s="12" t="inlineStr">
+        <is>
+          <t>COMMODITY</t>
+        </is>
+      </c>
+      <c r="F79" s="13" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G79" s="14" t="n">
+        <v>6.0055</v>
+      </c>
+      <c r="H79" s="14" t="inlineStr"/>
+      <c r="I79" s="12" t="n">
+        <v>488</v>
+      </c>
+      <c r="J79" s="14" t="n">
+        <v>2930.68</v>
+      </c>
+      <c r="K79" s="14" t="n">
+        <v>5.8554</v>
+      </c>
+      <c r="L79" s="14" t="n">
+        <v>6.1857</v>
+      </c>
+      <c r="M79" s="14" t="inlineStr"/>
+      <c r="N79" s="12" t="inlineStr"/>
+      <c r="O79" s="12" t="n">
+        <v>26.42</v>
+      </c>
+      <c r="P79" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q79" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R79" s="12" t="inlineStr">
+        <is>
+          <t>RSI BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="22" customHeight="1">
+      <c r="A80" s="15" t="n">
+        <v>78</v>
+      </c>
+      <c r="B80" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="C80" s="15" t="inlineStr">
+        <is>
+          <t>10:32</t>
+        </is>
+      </c>
+      <c r="D80" s="15" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="E80" s="15" t="inlineStr">
+        <is>
+          <t>COMMODITY</t>
+        </is>
+      </c>
+      <c r="F80" s="13" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G80" s="16" t="n">
+        <v>74.255</v>
+      </c>
+      <c r="H80" s="16" t="inlineStr"/>
+      <c r="I80" s="15" t="n">
+        <v>38</v>
+      </c>
+      <c r="J80" s="16" t="n">
+        <v>2821.69</v>
+      </c>
+      <c r="K80" s="16" t="n">
+        <v>72.3986</v>
+      </c>
+      <c r="L80" s="16" t="n">
+        <v>76.48260000000001</v>
+      </c>
+      <c r="M80" s="16" t="inlineStr"/>
+      <c r="N80" s="15" t="inlineStr"/>
+      <c r="O80" s="15" t="n">
+        <v>28.3</v>
+      </c>
+      <c r="P80" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q80" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="R80" s="15" t="inlineStr">
+        <is>
+          <t>RSI BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="22" customHeight="1">
+      <c r="A81" s="12" t="n">
+        <v>79</v>
+      </c>
+      <c r="B81" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="C81" s="12" t="inlineStr">
+        <is>
+          <t>13:19</t>
+        </is>
+      </c>
+      <c r="D81" s="12" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="E81" s="12" t="inlineStr">
+        <is>
+          <t>COMMODITY</t>
+        </is>
+      </c>
+      <c r="F81" s="13" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G81" s="14" t="n">
+        <v>4597.2998</v>
+      </c>
+      <c r="H81" s="14" t="inlineStr"/>
+      <c r="I81" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J81" s="14" t="n">
+        <v>4597.3</v>
+      </c>
+      <c r="K81" s="14" t="n">
+        <v>4482.3673</v>
+      </c>
+      <c r="L81" s="14" t="n">
+        <v>4735.2188</v>
+      </c>
+      <c r="M81" s="14" t="inlineStr"/>
+      <c r="N81" s="12" t="inlineStr"/>
+      <c r="O81" s="12" t="n">
+        <v>27.95</v>
+      </c>
+      <c r="P81" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q81" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R81" s="12" t="inlineStr">
+        <is>
+          <t>RSI BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="22" customHeight="1">
+      <c r="A82" s="15" t="n">
+        <v>80</v>
+      </c>
+      <c r="B82" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="C82" s="15" t="inlineStr">
+        <is>
+          <t>13:19</t>
+        </is>
+      </c>
+      <c r="D82" s="15" t="inlineStr">
+        <is>
+          <t>BZ</t>
+        </is>
+      </c>
+      <c r="E82" s="15" t="inlineStr">
+        <is>
+          <t>COMMODITY</t>
+        </is>
+      </c>
+      <c r="F82" s="13" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G82" s="16" t="n">
+        <v>104.09</v>
+      </c>
+      <c r="H82" s="16" t="inlineStr"/>
+      <c r="I82" s="15" t="n">
+        <v>25</v>
+      </c>
+      <c r="J82" s="16" t="n">
+        <v>2602.25</v>
+      </c>
+      <c r="K82" s="16" t="n">
+        <v>101.4878</v>
+      </c>
+      <c r="L82" s="16" t="n">
+        <v>107.2127</v>
+      </c>
+      <c r="M82" s="16" t="inlineStr"/>
+      <c r="N82" s="15" t="inlineStr"/>
+      <c r="O82" s="15" t="n">
+        <v>9.25</v>
+      </c>
+      <c r="P82" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q82" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="R82" s="15" t="inlineStr">
         <is>
           <t>RSI BUY</t>
         </is>
@@ -4938,7 +5795,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -5010,6 +5867,150 @@
         <is>
           <t>Worst ₹</t>
         </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="19" t="inlineStr">
+        <is>
+          <t>CRYPTO</t>
+        </is>
+      </c>
+      <c r="B3" s="19" t="inlineStr">
+        <is>
+          <t>AAVE-USD</t>
+        </is>
+      </c>
+      <c r="C3" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="21" t="n">
+        <v>-7826.1</v>
+      </c>
+      <c r="H3" s="21" t="n">
+        <v>-7826.1</v>
+      </c>
+      <c r="I3" s="21" t="n">
+        <v>-7826.1</v>
+      </c>
+      <c r="J3" s="21" t="n">
+        <v>-7826.1</v>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="19" t="inlineStr">
+        <is>
+          <t>CRYPTO</t>
+        </is>
+      </c>
+      <c r="B4" s="19" t="inlineStr">
+        <is>
+          <t>BNB-USD</t>
+        </is>
+      </c>
+      <c r="C4" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="F4" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="21" t="n">
+        <v>-104124.54</v>
+      </c>
+      <c r="H4" s="21" t="n">
+        <v>-52062.27</v>
+      </c>
+      <c r="I4" s="21" t="n">
+        <v>-52062.27</v>
+      </c>
+      <c r="J4" s="21" t="n">
+        <v>-52062.27</v>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="19" t="inlineStr">
+        <is>
+          <t>CRYPTO</t>
+        </is>
+      </c>
+      <c r="B5" s="19" t="inlineStr">
+        <is>
+          <t>LINK-USD</t>
+        </is>
+      </c>
+      <c r="C5" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="21" t="n">
+        <v>-4600.28</v>
+      </c>
+      <c r="H5" s="21" t="n">
+        <v>-2300.14</v>
+      </c>
+      <c r="I5" s="21" t="n">
+        <v>-2300.14</v>
+      </c>
+      <c r="J5" s="21" t="n">
+        <v>-2300.14</v>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="19" t="inlineStr">
+        <is>
+          <t>CRYPTO</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>SOL-USD</t>
+        </is>
+      </c>
+      <c r="C6" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="21" t="n">
+        <v>-13997.12</v>
+      </c>
+      <c r="H6" s="21" t="n">
+        <v>-6998.56</v>
+      </c>
+      <c r="I6" s="21" t="n">
+        <v>-6998.56</v>
+      </c>
+      <c r="J6" s="21" t="n">
+        <v>-6998.56</v>
       </c>
     </row>
   </sheetData>
@@ -5061,7 +6062,7 @@
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>₹89,441.45</t>
+          <t>₹84,747.35</t>
         </is>
       </c>
     </row>
@@ -5073,7 +6074,7 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>₹251.61</t>
+          <t>₹-138,374.14</t>
         </is>
       </c>
     </row>
@@ -5085,7 +6086,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>₹182.20</t>
+          <t>₹0.00</t>
         </is>
       </c>
     </row>
@@ -5097,7 +6098,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>₹89,623.65</t>
+          <t>₹84,747.35</t>
         </is>
       </c>
     </row>
@@ -5109,7 +6110,7 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>0.18%</t>
+          <t>0.0%</t>
         </is>
       </c>
     </row>
@@ -5120,7 +6121,7 @@
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
@@ -5130,7 +6131,7 @@
         </is>
       </c>
       <c r="B10" s="11" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
@@ -5140,7 +6141,7 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
@@ -5151,7 +6152,7 @@
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
     </row>
@@ -5174,7 +6175,7 @@
         </is>
       </c>
       <c r="B14" s="11" t="n">
-        <v>44.37</v>
+        <v>-7.7</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
@@ -5185,7 +6186,7 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>29-Apr-2026 09:20</t>
+          <t>01-May-2026 13:19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add telegram test script
</commit_message>
<xml_diff>
--- a/logs/Trading_Journal.xlsx
+++ b/logs/Trading_Journal.xlsx
@@ -593,7 +593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R82"/>
+  <dimension ref="A1:R83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5686,6 +5686,68 @@
         <v>0</v>
       </c>
       <c r="R82" s="15" t="inlineStr">
+        <is>
+          <t>RSI BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="22" customHeight="1">
+      <c r="A83" s="12" t="n">
+        <v>81</v>
+      </c>
+      <c r="B83" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="C83" s="12" t="inlineStr">
+        <is>
+          <t>13:34</t>
+        </is>
+      </c>
+      <c r="D83" s="12" t="inlineStr">
+        <is>
+          <t>TCS</t>
+        </is>
+      </c>
+      <c r="E83" s="12" t="inlineStr">
+        <is>
+          <t>STOCK</t>
+        </is>
+      </c>
+      <c r="F83" s="13" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G83" s="14" t="n">
+        <v>2426</v>
+      </c>
+      <c r="H83" s="14" t="inlineStr"/>
+      <c r="I83" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J83" s="14" t="n">
+        <v>2426</v>
+      </c>
+      <c r="K83" s="14" t="n">
+        <v>2377.48</v>
+      </c>
+      <c r="L83" s="14" t="n">
+        <v>2498.78</v>
+      </c>
+      <c r="M83" s="14" t="inlineStr"/>
+      <c r="N83" s="12" t="inlineStr"/>
+      <c r="O83" s="12" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="P83" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q83" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R83" s="12" t="inlineStr">
         <is>
           <t>RSI BUY</t>
         </is>
@@ -6062,7 +6124,7 @@
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>₹84,747.35</t>
+          <t>₹91,917.40</t>
         </is>
       </c>
     </row>
@@ -6074,7 +6136,7 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>₹-138,374.14</t>
+          <t>₹0.00</t>
         </is>
       </c>
     </row>
@@ -6098,7 +6160,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>₹84,747.35</t>
+          <t>₹91,917.40</t>
         </is>
       </c>
     </row>
@@ -6110,7 +6172,7 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>-8.08%</t>
         </is>
       </c>
     </row>
@@ -6121,7 +6183,7 @@
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
@@ -6141,7 +6203,7 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
@@ -6152,7 +6214,7 @@
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0%</t>
         </is>
       </c>
     </row>
@@ -6174,8 +6236,10 @@
           <t>Sharpe Ratio</t>
         </is>
       </c>
-      <c r="B14" s="11" t="n">
-        <v>-7.7</v>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
@@ -6186,7 +6250,7 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>01-May-2026 13:19</t>
+          <t>04-May-2026 13:34</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: dashboard capital display, orphaned JS removed, blueprint registered
</commit_message>
<xml_diff>
--- a/logs/Trading_Journal.xlsx
+++ b/logs/Trading_Journal.xlsx
@@ -70,7 +70,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -132,6 +132,11 @@
         <fgColor rgb="00E8F8F5"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDEDEC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -159,7 +164,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -225,6 +230,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -593,7 +610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R83"/>
+  <dimension ref="A1:R88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5753,6 +5770,332 @@
         </is>
       </c>
     </row>
+    <row r="84" ht="22" customHeight="1">
+      <c r="A84" s="15" t="n">
+        <v>82</v>
+      </c>
+      <c r="B84" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="C84" s="15" t="inlineStr">
+        <is>
+          <t>12:01</t>
+        </is>
+      </c>
+      <c r="D84" s="15" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="E84" s="15" t="inlineStr">
+        <is>
+          <t>US_STOCK</t>
+        </is>
+      </c>
+      <c r="F84" s="17" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="G84" s="16" t="n">
+        <v>26678.68</v>
+      </c>
+      <c r="H84" s="16" t="n">
+        <v>26363.4729</v>
+      </c>
+      <c r="I84" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="J84" s="16" t="n">
+        <v>266786.8</v>
+      </c>
+      <c r="K84" s="16" t="inlineStr"/>
+      <c r="L84" s="16" t="inlineStr"/>
+      <c r="M84" s="22" t="n">
+        <v>-3152.07</v>
+      </c>
+      <c r="N84" s="17" t="inlineStr">
+        <is>
+          <t>LOSS 🔴</t>
+        </is>
+      </c>
+      <c r="O84" s="15" t="n">
+        <v>50</v>
+      </c>
+      <c r="P84" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q84" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="R84" s="15" t="inlineStr">
+        <is>
+          <t>STOP-LOSS (-99.0%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="22" customHeight="1">
+      <c r="A85" s="12" t="n">
+        <v>83</v>
+      </c>
+      <c r="B85" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="C85" s="12" t="inlineStr">
+        <is>
+          <t>12:01</t>
+        </is>
+      </c>
+      <c r="D85" s="12" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="E85" s="12" t="inlineStr">
+        <is>
+          <t>US_STOCK</t>
+        </is>
+      </c>
+      <c r="F85" s="17" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="G85" s="14" t="n">
+        <v>8770.68</v>
+      </c>
+      <c r="H85" s="14" t="n">
+        <v>8669.739299999999</v>
+      </c>
+      <c r="I85" s="12" t="n">
+        <v>31</v>
+      </c>
+      <c r="J85" s="14" t="n">
+        <v>271891.08</v>
+      </c>
+      <c r="K85" s="14" t="inlineStr"/>
+      <c r="L85" s="14" t="inlineStr"/>
+      <c r="M85" s="18" t="n">
+        <v>-3129.16</v>
+      </c>
+      <c r="N85" s="17" t="inlineStr">
+        <is>
+          <t>LOSS 🔴</t>
+        </is>
+      </c>
+      <c r="O85" s="12" t="n">
+        <v>50</v>
+      </c>
+      <c r="P85" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q85" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R85" s="12" t="inlineStr">
+        <is>
+          <t>STOP-LOSS (-99.0%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="22" customHeight="1">
+      <c r="A86" s="15" t="n">
+        <v>84</v>
+      </c>
+      <c r="B86" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="C86" s="15" t="inlineStr">
+        <is>
+          <t>12:07</t>
+        </is>
+      </c>
+      <c r="D86" s="15" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="E86" s="15" t="inlineStr">
+        <is>
+          <t>US_STOCK</t>
+        </is>
+      </c>
+      <c r="F86" s="17" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="G86" s="16" t="n">
+        <v>26678.68</v>
+      </c>
+      <c r="H86" s="16" t="n">
+        <v>26363.4729</v>
+      </c>
+      <c r="I86" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="J86" s="16" t="n">
+        <v>266786.8</v>
+      </c>
+      <c r="K86" s="16" t="inlineStr"/>
+      <c r="L86" s="16" t="inlineStr"/>
+      <c r="M86" s="22" t="n">
+        <v>-3152.07</v>
+      </c>
+      <c r="N86" s="17" t="inlineStr">
+        <is>
+          <t>LOSS 🔴</t>
+        </is>
+      </c>
+      <c r="O86" s="15" t="n">
+        <v>50</v>
+      </c>
+      <c r="P86" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q86" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="R86" s="15" t="inlineStr">
+        <is>
+          <t>STOP-LOSS (-99.0%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="22" customHeight="1">
+      <c r="A87" s="12" t="n">
+        <v>85</v>
+      </c>
+      <c r="B87" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="C87" s="12" t="inlineStr">
+        <is>
+          <t>12:07</t>
+        </is>
+      </c>
+      <c r="D87" s="12" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="E87" s="12" t="inlineStr">
+        <is>
+          <t>US_STOCK</t>
+        </is>
+      </c>
+      <c r="F87" s="17" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="G87" s="14" t="n">
+        <v>8770.68</v>
+      </c>
+      <c r="H87" s="14" t="n">
+        <v>8669.739299999999</v>
+      </c>
+      <c r="I87" s="12" t="n">
+        <v>31</v>
+      </c>
+      <c r="J87" s="14" t="n">
+        <v>271891.08</v>
+      </c>
+      <c r="K87" s="14" t="inlineStr"/>
+      <c r="L87" s="14" t="inlineStr"/>
+      <c r="M87" s="18" t="n">
+        <v>-3129.16</v>
+      </c>
+      <c r="N87" s="17" t="inlineStr">
+        <is>
+          <t>LOSS 🔴</t>
+        </is>
+      </c>
+      <c r="O87" s="12" t="n">
+        <v>50</v>
+      </c>
+      <c r="P87" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q87" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R87" s="12" t="inlineStr">
+        <is>
+          <t>STOP-LOSS (-99.0%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="22" customHeight="1">
+      <c r="A88" s="15" t="n">
+        <v>86</v>
+      </c>
+      <c r="B88" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="C88" s="15" t="inlineStr">
+        <is>
+          <t>12:09</t>
+        </is>
+      </c>
+      <c r="D88" s="15" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="E88" s="15" t="inlineStr">
+        <is>
+          <t>STOCK</t>
+        </is>
+      </c>
+      <c r="F88" s="13" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G88" s="16" t="n">
+        <v>1248.9</v>
+      </c>
+      <c r="H88" s="16" t="inlineStr"/>
+      <c r="I88" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="J88" s="16" t="n">
+        <v>4995.6</v>
+      </c>
+      <c r="K88" s="16" t="n">
+        <v>1223.922</v>
+      </c>
+      <c r="L88" s="16" t="n">
+        <v>1286.367</v>
+      </c>
+      <c r="M88" s="16" t="inlineStr"/>
+      <c r="N88" s="15" t="inlineStr"/>
+      <c r="O88" s="15" t="n">
+        <v>40.69</v>
+      </c>
+      <c r="P88" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q88" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="R88" s="15" t="inlineStr">
+        <is>
+          <t>RSI BUY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:R1"/>
@@ -5768,7 +6111,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -5841,6 +6184,38 @@
           <t>Notes</t>
         </is>
       </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="B3" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="18" t="n">
+        <v>-6281.23</v>
+      </c>
+      <c r="G3" s="14" t="n">
+        <v>-6281.23</v>
+      </c>
+      <c r="H3" s="14" t="n">
+        <v>620345.65</v>
+      </c>
+      <c r="I3" s="14" t="n">
+        <v>-3129.16</v>
+      </c>
+      <c r="J3" s="12" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -5932,148 +6307,100 @@
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="19" t="inlineStr">
-        <is>
-          <t>CRYPTO</t>
-        </is>
-      </c>
-      <c r="B3" s="19" t="inlineStr">
-        <is>
-          <t>AAVE-USD</t>
-        </is>
-      </c>
-      <c r="C3" s="19" t="n">
+      <c r="A3" s="24" t="inlineStr">
+        <is>
+          <t>US_STOCK</t>
+        </is>
+      </c>
+      <c r="B3" s="24" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C3" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="D3" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" s="19" t="n">
+      <c r="D3" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="F3" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" s="21" t="n">
-        <v>-7826.1</v>
-      </c>
-      <c r="H3" s="21" t="n">
-        <v>-7826.1</v>
-      </c>
-      <c r="I3" s="21" t="n">
-        <v>-7826.1</v>
-      </c>
-      <c r="J3" s="21" t="n">
-        <v>-7826.1</v>
+      <c r="F3" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="26" t="n">
+        <v>-3152.07</v>
+      </c>
+      <c r="H3" s="26" t="n">
+        <v>-3152.07</v>
+      </c>
+      <c r="I3" s="26" t="n">
+        <v>-3152.07</v>
+      </c>
+      <c r="J3" s="26" t="n">
+        <v>-3152.07</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="19" t="inlineStr">
-        <is>
-          <t>CRYPTO</t>
-        </is>
-      </c>
-      <c r="B4" s="19" t="inlineStr">
-        <is>
-          <t>BNB-USD</t>
-        </is>
-      </c>
-      <c r="C4" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="D4" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="F4" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" s="21" t="n">
-        <v>-104124.54</v>
-      </c>
-      <c r="H4" s="21" t="n">
-        <v>-52062.27</v>
-      </c>
-      <c r="I4" s="21" t="n">
-        <v>-52062.27</v>
-      </c>
-      <c r="J4" s="21" t="n">
-        <v>-52062.27</v>
+      <c r="A4" s="24" t="inlineStr">
+        <is>
+          <t>US_STOCK</t>
+        </is>
+      </c>
+      <c r="B4" s="24" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="C4" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="26" t="n">
+        <v>-3129.16</v>
+      </c>
+      <c r="H4" s="26" t="n">
+        <v>-3129.16</v>
+      </c>
+      <c r="I4" s="26" t="n">
+        <v>-3129.16</v>
+      </c>
+      <c r="J4" s="26" t="n">
+        <v>-3129.16</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="19" t="inlineStr">
-        <is>
-          <t>CRYPTO</t>
-        </is>
-      </c>
-      <c r="B5" s="19" t="inlineStr">
-        <is>
-          <t>LINK-USD</t>
-        </is>
-      </c>
-      <c r="C5" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="D5" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="F5" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" s="21" t="n">
-        <v>-4600.28</v>
-      </c>
-      <c r="H5" s="21" t="n">
-        <v>-2300.14</v>
-      </c>
-      <c r="I5" s="21" t="n">
-        <v>-2300.14</v>
-      </c>
-      <c r="J5" s="21" t="n">
-        <v>-2300.14</v>
-      </c>
+      <c r="A5" s="19" t="n"/>
+      <c r="B5" s="19" t="n"/>
+      <c r="C5" s="19" t="n"/>
+      <c r="D5" s="19" t="n"/>
+      <c r="E5" s="19" t="n"/>
+      <c r="F5" s="20" t="n"/>
+      <c r="G5" s="21" t="n"/>
+      <c r="H5" s="21" t="n"/>
+      <c r="I5" s="21" t="n"/>
+      <c r="J5" s="21" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="19" t="inlineStr">
-        <is>
-          <t>CRYPTO</t>
-        </is>
-      </c>
-      <c r="B6" s="19" t="inlineStr">
-        <is>
-          <t>SOL-USD</t>
-        </is>
-      </c>
-      <c r="C6" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="D6" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="F6" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="21" t="n">
-        <v>-13997.12</v>
-      </c>
-      <c r="H6" s="21" t="n">
-        <v>-6998.56</v>
-      </c>
-      <c r="I6" s="21" t="n">
-        <v>-6998.56</v>
-      </c>
-      <c r="J6" s="21" t="n">
-        <v>-6998.56</v>
-      </c>
+      <c r="A6" s="19" t="n"/>
+      <c r="B6" s="19" t="n"/>
+      <c r="C6" s="19" t="n"/>
+      <c r="D6" s="19" t="n"/>
+      <c r="E6" s="19" t="n"/>
+      <c r="F6" s="20" t="n"/>
+      <c r="G6" s="21" t="n"/>
+      <c r="H6" s="21" t="n"/>
+      <c r="I6" s="21" t="n"/>
+      <c r="J6" s="21" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -6124,7 +6451,7 @@
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>₹91,917.40</t>
+          <t>₹615,350.05</t>
         </is>
       </c>
     </row>
@@ -6160,7 +6487,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>₹91,917.40</t>
+          <t>₹615,350.05</t>
         </is>
       </c>
     </row>
@@ -6172,7 +6499,7 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>-8.08%</t>
+          <t>515.35%</t>
         </is>
       </c>
     </row>
@@ -6250,7 +6577,7 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>04-May-2026 13:34</t>
+          <t>05-May-2026 12:09</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: wire Telegram alerts into paper_buy/paper_sell
</commit_message>
<xml_diff>
--- a/logs/Trading_Journal.xlsx
+++ b/logs/Trading_Journal.xlsx
@@ -610,7 +610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R88"/>
+  <dimension ref="A1:R89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6091,6 +6091,68 @@
         <v>0</v>
       </c>
       <c r="R88" s="15" t="inlineStr">
+        <is>
+          <t>RSI BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="22" customHeight="1">
+      <c r="A89" s="12" t="n">
+        <v>87</v>
+      </c>
+      <c r="B89" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="C89" s="12" t="inlineStr">
+        <is>
+          <t>12:53</t>
+        </is>
+      </c>
+      <c r="D89" s="12" t="inlineStr">
+        <is>
+          <t>ITC</t>
+        </is>
+      </c>
+      <c r="E89" s="12" t="inlineStr">
+        <is>
+          <t>STOCK</t>
+        </is>
+      </c>
+      <c r="F89" s="13" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G89" s="14" t="n">
+        <v>309.95</v>
+      </c>
+      <c r="H89" s="14" t="inlineStr"/>
+      <c r="I89" s="12" t="n">
+        <v>16</v>
+      </c>
+      <c r="J89" s="14" t="n">
+        <v>4959.2</v>
+      </c>
+      <c r="K89" s="14" t="n">
+        <v>303.751</v>
+      </c>
+      <c r="L89" s="14" t="n">
+        <v>319.2485</v>
+      </c>
+      <c r="M89" s="14" t="inlineStr"/>
+      <c r="N89" s="12" t="inlineStr"/>
+      <c r="O89" s="12" t="n">
+        <v>41.35</v>
+      </c>
+      <c r="P89" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q89" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R89" s="12" t="inlineStr">
         <is>
           <t>RSI BUY</t>
         </is>
@@ -6451,7 +6513,7 @@
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>₹615,350.05</t>
+          <t>₹344,025.38</t>
         </is>
       </c>
     </row>
@@ -6475,7 +6537,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>₹0.00</t>
+          <t>₹3,811.57</t>
         </is>
       </c>
     </row>
@@ -6487,7 +6549,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>₹615,350.05</t>
+          <t>₹347,836.96</t>
         </is>
       </c>
     </row>
@@ -6499,7 +6561,7 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>515.35%</t>
+          <t>247.84%</t>
         </is>
       </c>
     </row>
@@ -6577,7 +6639,7 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>05-May-2026 12:09</t>
+          <t>06-May-2026 12:53</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix: Telegram sell alert shows correct capital, recreated check_neon.py
</commit_message>
<xml_diff>
--- a/logs/Trading_Journal.xlsx
+++ b/logs/Trading_Journal.xlsx
@@ -164,7 +164,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -242,6 +242,21 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -610,7 +625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R89"/>
+  <dimension ref="A1:R90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6158,6 +6173,72 @@
         </is>
       </c>
     </row>
+    <row r="90" ht="22" customHeight="1">
+      <c r="A90" s="15" t="n">
+        <v>88</v>
+      </c>
+      <c r="B90" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C90" s="15" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="D90" s="15" t="inlineStr">
+        <is>
+          <t>SBIN</t>
+        </is>
+      </c>
+      <c r="E90" s="15" t="inlineStr">
+        <is>
+          <t>STOCK</t>
+        </is>
+      </c>
+      <c r="F90" s="17" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="G90" s="16" t="n">
+        <v>1069.4</v>
+      </c>
+      <c r="H90" s="16" t="n">
+        <v>1102.7</v>
+      </c>
+      <c r="I90" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="J90" s="16" t="n">
+        <v>2138.8</v>
+      </c>
+      <c r="K90" s="16" t="inlineStr"/>
+      <c r="L90" s="16" t="inlineStr"/>
+      <c r="M90" s="27" t="n">
+        <v>66.59999999999999</v>
+      </c>
+      <c r="N90" s="13" t="inlineStr">
+        <is>
+          <t>WIN 🟢</t>
+        </is>
+      </c>
+      <c r="O90" s="15" t="n">
+        <v>79.56999999999999</v>
+      </c>
+      <c r="P90" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q90" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="R90" s="15" t="inlineStr">
+        <is>
+          <t>TARGET HIT 🎯</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:R1"/>
@@ -6173,7 +6254,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -6278,6 +6359,38 @@
         <v>-3129.16</v>
       </c>
       <c r="J3" s="12" t="inlineStr"/>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="28" t="n">
+        <v>100</v>
+      </c>
+      <c r="F4" s="27" t="n">
+        <v>66.59999999999999</v>
+      </c>
+      <c r="G4" s="16" t="n">
+        <v>66.59999999999999</v>
+      </c>
+      <c r="H4" s="16" t="n">
+        <v>346230.78</v>
+      </c>
+      <c r="I4" s="16" t="n">
+        <v>66.59999999999999</v>
+      </c>
+      <c r="J4" s="15" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -6369,76 +6482,52 @@
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="24" t="inlineStr">
-        <is>
-          <t>US_STOCK</t>
-        </is>
-      </c>
-      <c r="B3" s="24" t="inlineStr">
-        <is>
-          <t>AAPL</t>
-        </is>
-      </c>
-      <c r="C3" s="24" t="n">
+      <c r="A3" s="29" t="inlineStr">
+        <is>
+          <t>STOCK</t>
+        </is>
+      </c>
+      <c r="B3" s="29" t="inlineStr">
+        <is>
+          <t>SBIN</t>
+        </is>
+      </c>
+      <c r="C3" s="29" t="n">
         <v>1</v>
       </c>
-      <c r="D3" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" s="24" t="n">
+      <c r="D3" s="29" t="n">
         <v>1</v>
       </c>
-      <c r="F3" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" s="26" t="n">
-        <v>-3152.07</v>
-      </c>
-      <c r="H3" s="26" t="n">
-        <v>-3152.07</v>
-      </c>
-      <c r="I3" s="26" t="n">
-        <v>-3152.07</v>
-      </c>
-      <c r="J3" s="26" t="n">
-        <v>-3152.07</v>
+      <c r="E3" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="30" t="n">
+        <v>100</v>
+      </c>
+      <c r="G3" s="31" t="n">
+        <v>66.59999999999999</v>
+      </c>
+      <c r="H3" s="31" t="n">
+        <v>66.59999999999999</v>
+      </c>
+      <c r="I3" s="31" t="n">
+        <v>66.59999999999999</v>
+      </c>
+      <c r="J3" s="31" t="n">
+        <v>66.59999999999999</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="24" t="inlineStr">
-        <is>
-          <t>US_STOCK</t>
-        </is>
-      </c>
-      <c r="B4" s="24" t="inlineStr">
-        <is>
-          <t>NFLX</t>
-        </is>
-      </c>
-      <c r="C4" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="F4" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" s="26" t="n">
-        <v>-3129.16</v>
-      </c>
-      <c r="H4" s="26" t="n">
-        <v>-3129.16</v>
-      </c>
-      <c r="I4" s="26" t="n">
-        <v>-3129.16</v>
-      </c>
-      <c r="J4" s="26" t="n">
-        <v>-3129.16</v>
-      </c>
+      <c r="A4" s="24" t="n"/>
+      <c r="B4" s="24" t="n"/>
+      <c r="C4" s="24" t="n"/>
+      <c r="D4" s="24" t="n"/>
+      <c r="E4" s="24" t="n"/>
+      <c r="F4" s="25" t="n"/>
+      <c r="G4" s="26" t="n"/>
+      <c r="H4" s="26" t="n"/>
+      <c r="I4" s="26" t="n"/>
+      <c r="J4" s="26" t="n"/>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="19" t="n"/>
@@ -6513,7 +6602,7 @@
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>₹344,025.38</t>
+          <t>₹346,230.78</t>
         </is>
       </c>
     </row>
@@ -6525,7 +6614,7 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>₹0.00</t>
+          <t>₹66.60</t>
         </is>
       </c>
     </row>
@@ -6537,7 +6626,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>₹3,811.57</t>
+          <t>₹7,074.84</t>
         </is>
       </c>
     </row>
@@ -6549,7 +6638,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>₹347,836.96</t>
+          <t>₹353,305.63</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6650,7 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>247.84%</t>
+          <t>253.31%</t>
         </is>
       </c>
     </row>
@@ -6572,7 +6661,7 @@
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
@@ -6582,7 +6671,7 @@
         </is>
       </c>
       <c r="B10" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
@@ -6603,7 +6692,7 @@
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100.0%</t>
         </is>
       </c>
     </row>
@@ -6639,7 +6728,7 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>06-May-2026 12:53</t>
+          <t>07-May-2026 09:15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Feature: Upstox positions + token persisted to Neon DB
</commit_message>
<xml_diff>
--- a/logs/Trading_Journal.xlsx
+++ b/logs/Trading_Journal.xlsx
@@ -625,7 +625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R90"/>
+  <dimension ref="A1:R91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6236,6 +6236,68 @@
       <c r="R90" s="15" t="inlineStr">
         <is>
           <t>TARGET HIT 🎯</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="22" customHeight="1">
+      <c r="A91" s="12" t="n">
+        <v>89</v>
+      </c>
+      <c r="B91" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="C91" s="12" t="inlineStr">
+        <is>
+          <t>10:38</t>
+        </is>
+      </c>
+      <c r="D91" s="12" t="inlineStr">
+        <is>
+          <t>MARUTI</t>
+        </is>
+      </c>
+      <c r="E91" s="12" t="inlineStr">
+        <is>
+          <t>STOCK</t>
+        </is>
+      </c>
+      <c r="F91" s="13" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G91" s="14" t="n">
+        <v>13684</v>
+      </c>
+      <c r="H91" s="14" t="inlineStr"/>
+      <c r="I91" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J91" s="14" t="n">
+        <v>13684</v>
+      </c>
+      <c r="K91" s="14" t="n">
+        <v>13410.32</v>
+      </c>
+      <c r="L91" s="14" t="n">
+        <v>14094.52</v>
+      </c>
+      <c r="M91" s="14" t="inlineStr"/>
+      <c r="N91" s="12" t="inlineStr"/>
+      <c r="O91" s="12" t="n">
+        <v>44.13</v>
+      </c>
+      <c r="P91" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q91" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R91" s="12" t="inlineStr">
+        <is>
+          <t>RSI BUY</t>
         </is>
       </c>
     </row>
@@ -6602,7 +6664,7 @@
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>₹346,230.78</t>
+          <t>₹315,097.96</t>
         </is>
       </c>
     </row>
@@ -6614,7 +6676,7 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>₹66.60</t>
+          <t>₹152.20</t>
         </is>
       </c>
     </row>
@@ -6626,7 +6688,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>₹7,074.84</t>
+          <t>₹1,957.39</t>
         </is>
       </c>
     </row>
@@ -6638,7 +6700,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>₹353,305.63</t>
+          <t>₹317,055.35</t>
         </is>
       </c>
     </row>
@@ -6650,7 +6712,7 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>253.31%</t>
+          <t>217.06%</t>
         </is>
       </c>
     </row>
@@ -6661,7 +6723,7 @@
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
@@ -6671,7 +6733,7 @@
         </is>
       </c>
       <c r="B10" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
@@ -6714,10 +6776,8 @@
           <t>Sharpe Ratio</t>
         </is>
       </c>
-      <c r="B14" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="B14" s="11" t="n">
+        <v>81.34999999999999</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
@@ -6728,7 +6788,7 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>07-May-2026 09:15</t>
+          <t>08-May-2026 10:39</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix: Remove button deletes by symbol+broker, not all rows
</commit_message>
<xml_diff>
--- a/logs/Trading_Journal.xlsx
+++ b/logs/Trading_Journal.xlsx
@@ -625,7 +625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R91"/>
+  <dimension ref="A1:R92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6296,6 +6296,68 @@
         <v>0</v>
       </c>
       <c r="R91" s="12" t="inlineStr">
+        <is>
+          <t>RSI BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="22" customHeight="1">
+      <c r="A92" s="15" t="n">
+        <v>90</v>
+      </c>
+      <c r="B92" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="C92" s="15" t="inlineStr">
+        <is>
+          <t>11:29</t>
+        </is>
+      </c>
+      <c r="D92" s="15" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="E92" s="15" t="inlineStr">
+        <is>
+          <t>STOCK</t>
+        </is>
+      </c>
+      <c r="F92" s="13" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G92" s="16" t="n">
+        <v>1764.3</v>
+      </c>
+      <c r="H92" s="16" t="inlineStr"/>
+      <c r="I92" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="J92" s="16" t="n">
+        <v>8821.5</v>
+      </c>
+      <c r="K92" s="16" t="n">
+        <v>1729.014</v>
+      </c>
+      <c r="L92" s="16" t="n">
+        <v>1817.229</v>
+      </c>
+      <c r="M92" s="16" t="inlineStr"/>
+      <c r="N92" s="15" t="inlineStr"/>
+      <c r="O92" s="15" t="n">
+        <v>21.33</v>
+      </c>
+      <c r="P92" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q92" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="R92" s="15" t="inlineStr">
         <is>
           <t>RSI BUY</t>
         </is>
@@ -6664,7 +6726,7 @@
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>₹315,097.96</t>
+          <t>₹297,482.16</t>
         </is>
       </c>
     </row>
@@ -6688,7 +6750,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>₹1,957.39</t>
+          <t>₹0.00</t>
         </is>
       </c>
     </row>
@@ -6700,7 +6762,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>₹317,055.35</t>
+          <t>₹297,482.16</t>
         </is>
       </c>
     </row>
@@ -6712,7 +6774,7 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>217.06%</t>
+          <t>197.48%</t>
         </is>
       </c>
     </row>
@@ -6788,7 +6850,7 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>08-May-2026 10:39</t>
+          <t>11-May-2026 11:29</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update logs, bot state and backtest script - 2026-05-12
</commit_message>
<xml_diff>
--- a/logs/Trading_Journal.xlsx
+++ b/logs/Trading_Journal.xlsx
@@ -625,7 +625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R92"/>
+  <dimension ref="A1:R95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6358,6 +6358,192 @@
         <v>0</v>
       </c>
       <c r="R92" s="15" t="inlineStr">
+        <is>
+          <t>RSI BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="22" customHeight="1">
+      <c r="A93" s="12" t="n">
+        <v>91</v>
+      </c>
+      <c r="B93" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="C93" s="12" t="inlineStr">
+        <is>
+          <t>10:43</t>
+        </is>
+      </c>
+      <c r="D93" s="12" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="E93" s="12" t="inlineStr">
+        <is>
+          <t>STOCK</t>
+        </is>
+      </c>
+      <c r="F93" s="13" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G93" s="14" t="n">
+        <v>1246.7</v>
+      </c>
+      <c r="H93" s="14" t="inlineStr"/>
+      <c r="I93" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="J93" s="14" t="n">
+        <v>8726.9</v>
+      </c>
+      <c r="K93" s="14" t="n">
+        <v>1221.766</v>
+      </c>
+      <c r="L93" s="14" t="n">
+        <v>1284.101</v>
+      </c>
+      <c r="M93" s="14" t="inlineStr"/>
+      <c r="N93" s="12" t="inlineStr"/>
+      <c r="O93" s="12" t="n">
+        <v>30.25</v>
+      </c>
+      <c r="P93" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q93" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R93" s="12" t="inlineStr">
+        <is>
+          <t>RSI BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="22" customHeight="1">
+      <c r="A94" s="15" t="n">
+        <v>92</v>
+      </c>
+      <c r="B94" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="C94" s="15" t="inlineStr">
+        <is>
+          <t>10:44</t>
+        </is>
+      </c>
+      <c r="D94" s="15" t="inlineStr">
+        <is>
+          <t>RELIANCE</t>
+        </is>
+      </c>
+      <c r="E94" s="15" t="inlineStr">
+        <is>
+          <t>STOCK</t>
+        </is>
+      </c>
+      <c r="F94" s="13" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G94" s="16" t="n">
+        <v>1382</v>
+      </c>
+      <c r="H94" s="16" t="inlineStr"/>
+      <c r="I94" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="J94" s="16" t="n">
+        <v>8292</v>
+      </c>
+      <c r="K94" s="16" t="n">
+        <v>1354.36</v>
+      </c>
+      <c r="L94" s="16" t="n">
+        <v>1423.46</v>
+      </c>
+      <c r="M94" s="16" t="inlineStr"/>
+      <c r="N94" s="15" t="inlineStr"/>
+      <c r="O94" s="15" t="n">
+        <v>36.22</v>
+      </c>
+      <c r="P94" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q94" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="R94" s="15" t="inlineStr">
+        <is>
+          <t>RSI BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="22" customHeight="1">
+      <c r="A95" s="12" t="n">
+        <v>93</v>
+      </c>
+      <c r="B95" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="C95" s="12" t="inlineStr">
+        <is>
+          <t>11:38</t>
+        </is>
+      </c>
+      <c r="D95" s="12" t="inlineStr">
+        <is>
+          <t>TCS</t>
+        </is>
+      </c>
+      <c r="E95" s="12" t="inlineStr">
+        <is>
+          <t>STOCK</t>
+        </is>
+      </c>
+      <c r="F95" s="13" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G95" s="14" t="n">
+        <v>2297.5</v>
+      </c>
+      <c r="H95" s="14" t="inlineStr"/>
+      <c r="I95" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="J95" s="14" t="n">
+        <v>6892.5</v>
+      </c>
+      <c r="K95" s="14" t="n">
+        <v>2251.55</v>
+      </c>
+      <c r="L95" s="14" t="n">
+        <v>2366.425</v>
+      </c>
+      <c r="M95" s="14" t="inlineStr"/>
+      <c r="N95" s="12" t="inlineStr"/>
+      <c r="O95" s="12" t="n">
+        <v>36.22</v>
+      </c>
+      <c r="P95" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q95" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R95" s="12" t="inlineStr">
         <is>
           <t>RSI BUY</t>
         </is>
@@ -6726,7 +6912,7 @@
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>₹297,482.16</t>
+          <t>₹291,772.56</t>
         </is>
       </c>
     </row>
@@ -6762,7 +6948,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>₹297,482.16</t>
+          <t>₹291,772.56</t>
         </is>
       </c>
     </row>
@@ -6774,7 +6960,7 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>197.48%</t>
+          <t>191.77%</t>
         </is>
       </c>
     </row>
@@ -6850,7 +7036,7 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>11-May-2026 11:29</t>
+          <t>12-May-2026 11:38</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 200MA trend filter to block downtrend entries
</commit_message>
<xml_diff>
--- a/logs/Trading_Journal.xlsx
+++ b/logs/Trading_Journal.xlsx
@@ -625,7 +625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R95"/>
+  <dimension ref="A1:R96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6544,6 +6544,68 @@
         <v>0</v>
       </c>
       <c r="R95" s="12" t="inlineStr">
+        <is>
+          <t>RSI BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="22" customHeight="1">
+      <c r="A96" s="15" t="n">
+        <v>94</v>
+      </c>
+      <c r="B96" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="C96" s="15" t="inlineStr">
+        <is>
+          <t>11:59</t>
+        </is>
+      </c>
+      <c r="D96" s="15" t="inlineStr">
+        <is>
+          <t>LT</t>
+        </is>
+      </c>
+      <c r="E96" s="15" t="inlineStr">
+        <is>
+          <t>STOCK</t>
+        </is>
+      </c>
+      <c r="F96" s="13" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G96" s="16" t="n">
+        <v>3895</v>
+      </c>
+      <c r="H96" s="16" t="inlineStr"/>
+      <c r="I96" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="J96" s="16" t="n">
+        <v>7790</v>
+      </c>
+      <c r="K96" s="16" t="n">
+        <v>3817.1</v>
+      </c>
+      <c r="L96" s="16" t="n">
+        <v>4011.85</v>
+      </c>
+      <c r="M96" s="16" t="inlineStr"/>
+      <c r="N96" s="15" t="inlineStr"/>
+      <c r="O96" s="15" t="n">
+        <v>36.85</v>
+      </c>
+      <c r="P96" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q96" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="R96" s="15" t="inlineStr">
         <is>
           <t>RSI BUY</t>
         </is>
@@ -6912,7 +6974,7 @@
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>₹291,772.56</t>
+          <t>₹290,875.06</t>
         </is>
       </c>
     </row>
@@ -6948,7 +7010,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>₹291,772.56</t>
+          <t>₹290,875.06</t>
         </is>
       </c>
     </row>
@@ -6960,7 +7022,7 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>191.77%</t>
+          <t>190.88%</t>
         </is>
       </c>
     </row>
@@ -7036,7 +7098,7 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>12-May-2026 11:38</t>
+          <t>12-May-2026 11:59</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix: Telegram 3 channel routing — Buy/Sell/System alerts separated
</commit_message>
<xml_diff>
--- a/logs/Trading_Journal.xlsx
+++ b/logs/Trading_Journal.xlsx
@@ -164,7 +164,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -257,6 +257,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -625,7 +628,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R96"/>
+  <dimension ref="A1:R97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6611,6 +6614,72 @@
         </is>
       </c>
     </row>
+    <row r="97" ht="22" customHeight="1">
+      <c r="A97" s="12" t="n">
+        <v>95</v>
+      </c>
+      <c r="B97" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="C97" s="12" t="inlineStr">
+        <is>
+          <t>09:51</t>
+        </is>
+      </c>
+      <c r="D97" s="12" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="E97" s="12" t="inlineStr">
+        <is>
+          <t>STOCK</t>
+        </is>
+      </c>
+      <c r="F97" s="17" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="G97" s="14" t="n">
+        <v>1764.3</v>
+      </c>
+      <c r="H97" s="14" t="n">
+        <v>1827.5</v>
+      </c>
+      <c r="I97" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="J97" s="14" t="n">
+        <v>8821.5</v>
+      </c>
+      <c r="K97" s="14" t="inlineStr"/>
+      <c r="L97" s="14" t="inlineStr"/>
+      <c r="M97" s="32" t="n">
+        <v>316</v>
+      </c>
+      <c r="N97" s="13" t="inlineStr">
+        <is>
+          <t>WIN 🟢</t>
+        </is>
+      </c>
+      <c r="O97" s="12" t="n">
+        <v>80.7</v>
+      </c>
+      <c r="P97" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q97" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R97" s="12" t="inlineStr">
+        <is>
+          <t>TARGET HIT 🎯</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:R1"/>
@@ -6626,7 +6695,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -6763,6 +6832,38 @@
         <v>66.59999999999999</v>
       </c>
       <c r="J4" s="15" t="inlineStr"/>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="23" t="n">
+        <v>100</v>
+      </c>
+      <c r="F5" s="32" t="n">
+        <v>316</v>
+      </c>
+      <c r="G5" s="14" t="n">
+        <v>468.2</v>
+      </c>
+      <c r="H5" s="14" t="n">
+        <v>306992.01</v>
+      </c>
+      <c r="I5" s="14" t="n">
+        <v>316</v>
+      </c>
+      <c r="J5" s="12" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -6861,7 +6962,7 @@
       </c>
       <c r="B3" s="29" t="inlineStr">
         <is>
-          <t>SBIN</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="C3" s="29" t="n">
@@ -6877,41 +6978,89 @@
         <v>100</v>
       </c>
       <c r="G3" s="31" t="n">
-        <v>66.59999999999999</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="H3" s="31" t="n">
-        <v>66.59999999999999</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="I3" s="31" t="n">
-        <v>66.59999999999999</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="J3" s="31" t="n">
-        <v>66.59999999999999</v>
+        <v>86.59999999999999</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="24" t="n"/>
-      <c r="B4" s="24" t="n"/>
-      <c r="C4" s="24" t="n"/>
-      <c r="D4" s="24" t="n"/>
-      <c r="E4" s="24" t="n"/>
-      <c r="F4" s="25" t="n"/>
-      <c r="G4" s="26" t="n"/>
-      <c r="H4" s="26" t="n"/>
-      <c r="I4" s="26" t="n"/>
-      <c r="J4" s="26" t="n"/>
+      <c r="A4" s="29" t="inlineStr">
+        <is>
+          <t>STOCK</t>
+        </is>
+      </c>
+      <c r="B4" s="29" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="C4" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="30" t="n">
+        <v>100</v>
+      </c>
+      <c r="G4" s="31" t="n">
+        <v>316</v>
+      </c>
+      <c r="H4" s="31" t="n">
+        <v>316</v>
+      </c>
+      <c r="I4" s="31" t="n">
+        <v>316</v>
+      </c>
+      <c r="J4" s="31" t="n">
+        <v>316</v>
+      </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="19" t="n"/>
-      <c r="B5" s="19" t="n"/>
-      <c r="C5" s="19" t="n"/>
-      <c r="D5" s="19" t="n"/>
-      <c r="E5" s="19" t="n"/>
-      <c r="F5" s="20" t="n"/>
-      <c r="G5" s="21" t="n"/>
-      <c r="H5" s="21" t="n"/>
-      <c r="I5" s="21" t="n"/>
-      <c r="J5" s="21" t="n"/>
+      <c r="A5" s="29" t="inlineStr">
+        <is>
+          <t>STOCK</t>
+        </is>
+      </c>
+      <c r="B5" s="29" t="inlineStr">
+        <is>
+          <t>SBIN</t>
+        </is>
+      </c>
+      <c r="C5" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="30" t="n">
+        <v>100</v>
+      </c>
+      <c r="G5" s="31" t="n">
+        <v>65.59999999999999</v>
+      </c>
+      <c r="H5" s="31" t="n">
+        <v>65.59999999999999</v>
+      </c>
+      <c r="I5" s="31" t="n">
+        <v>65.59999999999999</v>
+      </c>
+      <c r="J5" s="31" t="n">
+        <v>65.59999999999999</v>
+      </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="19" t="n"/>
@@ -6974,7 +7123,7 @@
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>₹290,875.06</t>
+          <t>₹306,992.01</t>
         </is>
       </c>
     </row>
@@ -6986,7 +7135,7 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>₹152.20</t>
+          <t>₹468.20</t>
         </is>
       </c>
     </row>
@@ -6998,7 +7147,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>₹0.00</t>
+          <t>₹75.78</t>
         </is>
       </c>
     </row>
@@ -7010,7 +7159,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>₹290,875.06</t>
+          <t>₹307,067.79</t>
         </is>
       </c>
     </row>
@@ -7022,7 +7171,7 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>190.88%</t>
+          <t>207.07%</t>
         </is>
       </c>
     </row>
@@ -7033,7 +7182,7 @@
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
@@ -7043,7 +7192,7 @@
         </is>
       </c>
       <c r="B10" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
@@ -7087,7 +7236,7 @@
         </is>
       </c>
       <c r="B14" s="11" t="n">
-        <v>81.34999999999999</v>
+        <v>17.84</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
@@ -7098,7 +7247,7 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>12-May-2026 11:59</t>
+          <t>14-May-2026 09:51</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Restore run_scheduler, add monitor_sl auto-SL-close every 5 min
</commit_message>
<xml_diff>
--- a/logs/Trading_Journal.xlsx
+++ b/logs/Trading_Journal.xlsx
@@ -628,7 +628,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R97"/>
+  <dimension ref="A1:R98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6677,6 +6677,68 @@
       <c r="R97" s="12" t="inlineStr">
         <is>
           <t>TARGET HIT 🎯</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="22" customHeight="1">
+      <c r="A98" s="15" t="n">
+        <v>96</v>
+      </c>
+      <c r="B98" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="C98" s="15" t="inlineStr">
+        <is>
+          <t>12:14</t>
+        </is>
+      </c>
+      <c r="D98" s="15" t="inlineStr">
+        <is>
+          <t>NTPC</t>
+        </is>
+      </c>
+      <c r="E98" s="15" t="inlineStr">
+        <is>
+          <t>STOCK</t>
+        </is>
+      </c>
+      <c r="F98" s="13" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G98" s="16" t="n">
+        <v>393.45</v>
+      </c>
+      <c r="H98" s="16" t="inlineStr"/>
+      <c r="I98" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="J98" s="16" t="n">
+        <v>6295.2</v>
+      </c>
+      <c r="K98" s="16" t="n">
+        <v>385.581</v>
+      </c>
+      <c r="L98" s="16" t="n">
+        <v>405.2535</v>
+      </c>
+      <c r="M98" s="16" t="inlineStr"/>
+      <c r="N98" s="15" t="inlineStr"/>
+      <c r="O98" s="15" t="n">
+        <v>39.8</v>
+      </c>
+      <c r="P98" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q98" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="R98" s="15" t="inlineStr">
+        <is>
+          <t>RSI BUY</t>
         </is>
       </c>
     </row>
@@ -7123,7 +7185,7 @@
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>₹306,992.01</t>
+          <t>₹309,625.41</t>
         </is>
       </c>
     </row>
@@ -7135,7 +7197,7 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>₹468.20</t>
+          <t>₹455.05</t>
         </is>
       </c>
     </row>
@@ -7147,7 +7209,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>₹75.78</t>
+          <t>₹-71.00</t>
         </is>
       </c>
     </row>
@@ -7159,7 +7221,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>₹307,067.79</t>
+          <t>₹309,554.41</t>
         </is>
       </c>
     </row>
@@ -7171,7 +7233,7 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>207.07%</t>
+          <t>209.55%</t>
         </is>
       </c>
     </row>
@@ -7182,7 +7244,7 @@
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
@@ -7192,7 +7254,7 @@
         </is>
       </c>
       <c r="B10" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
@@ -7236,7 +7298,7 @@
         </is>
       </c>
       <c r="B14" s="11" t="n">
-        <v>17.84</v>
+        <v>16.17</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
@@ -7247,7 +7309,7 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>14-May-2026 09:51</t>
+          <t>15-May-2026 12:14</t>
         </is>
       </c>
     </row>

</xml_diff>